<commit_message>
Optimize UI responsiveness and scanning performance for V1.0 release
</commit_message>
<xml_diff>
--- a/reports/PII_Discovery_Report.xlsx
+++ b/reports/PII_Discovery_Report.xlsx
@@ -671,7 +671,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scan: 2026-07-28 11:19:22  |  Target: E:\projects\office_tool\Data_discovery\test  |  v3.0.0  |  NER: en_core_web_lg</t>
+          <t>Scan: 2026-07-29 13:21:34  |  Target: E:\projects\office_tool\Data_discovery\test  |  v3.0.0  |  NER: en_core_web_lg</t>
         </is>
       </c>
     </row>
@@ -6610,12 +6610,12 @@
       </c>
       <c r="C104" s="30" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D104" s="31" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
+          <t>XXXXXX8277</t>
         </is>
       </c>
       <c r="E104" s="32" t="inlineStr">
@@ -6635,17 +6635,17 @@
       </c>
       <c r="H104" s="30" t="inlineStr">
         <is>
-          <t>Line 1</t>
+          <t>Line 10</t>
         </is>
       </c>
       <c r="I104" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J104" s="31" t="inlineStr">
         <is>
-          <t>From:"Parmod Kumar" &lt;i***d@sportking.co.in&gt;</t>
+          <t>XXXXXX8277</t>
         </is>
       </c>
     </row>
@@ -6660,12 +6660,12 @@
       </c>
       <c r="C105" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D105" s="34" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
       <c r="E105" s="32" t="inlineStr">
@@ -6685,17 +6685,17 @@
       </c>
       <c r="H105" s="33" t="inlineStr">
         <is>
-          <t>Line 2</t>
+          <t>Line 21</t>
         </is>
       </c>
       <c r="I105" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J105" s="34" t="inlineStr">
         <is>
-          <t>To: "Rahul Raj" &lt;r***d@mawaimail.com&gt;</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
     </row>
@@ -6715,7 +6715,7 @@
       </c>
       <c r="D106" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8277</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
       <c r="E106" s="32" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="H106" s="30" t="inlineStr">
         <is>
-          <t>Line 10</t>
+          <t>Line 46</t>
         </is>
       </c>
       <c r="I106" s="31" t="inlineStr">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="J106" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8277</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
     </row>
@@ -6760,12 +6760,12 @@
       </c>
       <c r="C107" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D107" s="34" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>XXXXXX7531</t>
         </is>
       </c>
       <c r="E107" s="32" t="inlineStr">
@@ -6785,17 +6785,17 @@
       </c>
       <c r="H107" s="33" t="inlineStr">
         <is>
-          <t>Line 11</t>
+          <t>Line 61</t>
         </is>
       </c>
       <c r="I107" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J107" s="34" t="inlineStr">
         <is>
-          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>XXXXXX7531</t>
         </is>
       </c>
     </row>
@@ -6810,12 +6810,12 @@
       </c>
       <c r="C108" s="30" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D108" s="31" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
       <c r="E108" s="32" t="inlineStr">
@@ -6835,17 +6835,17 @@
       </c>
       <c r="H108" s="30" t="inlineStr">
         <is>
-          <t>Line 13</t>
+          <t>Line 78</t>
         </is>
       </c>
       <c r="I108" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J108" s="31" t="inlineStr">
         <is>
-          <t>To: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
     </row>
@@ -6860,12 +6860,12 @@
       </c>
       <c r="C109" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D109" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
       <c r="E109" s="32" t="inlineStr">
@@ -6885,17 +6885,17 @@
       </c>
       <c r="H109" s="33" t="inlineStr">
         <is>
-          <t>Line 14</t>
+          <t>Line 103</t>
         </is>
       </c>
       <c r="I109" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J109" s="34" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
     </row>
@@ -6910,12 +6910,12 @@
       </c>
       <c r="C110" s="30" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D110" s="31" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>XXXXXX8277</t>
         </is>
       </c>
       <c r="E110" s="32" t="inlineStr">
@@ -6935,17 +6935,17 @@
       </c>
       <c r="H110" s="30" t="inlineStr">
         <is>
-          <t>Line 14</t>
+          <t>Line 119</t>
         </is>
       </c>
       <c r="I110" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J110" s="31" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>XXXXXX8277</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="H111" s="33" t="inlineStr">
         <is>
-          <t>Line 21</t>
+          <t>Line 132</t>
         </is>
       </c>
       <c r="I111" s="34" t="inlineStr">
@@ -7010,22 +7010,22 @@
       </c>
       <c r="C112" s="30" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D112" s="31" t="inlineStr">
         <is>
-          <t>20XX07</t>
-        </is>
-      </c>
-      <c r="E112" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>XXXXXX8277</t>
+        </is>
+      </c>
+      <c r="E112" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F112" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G112" s="30" t="inlineStr">
@@ -7035,17 +7035,17 @@
       </c>
       <c r="H112" s="30" t="inlineStr">
         <is>
-          <t>Line 25</t>
+          <t>Line 156</t>
         </is>
       </c>
       <c r="I112" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J112" s="31" t="inlineStr">
         <is>
-          <t>20XX07- U.P</t>
+          <t>Phone Number XXXXXX8277</t>
         </is>
       </c>
     </row>
@@ -7060,12 +7060,12 @@
       </c>
       <c r="C113" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PHONE_IN</t>
         </is>
       </c>
       <c r="D113" s="34" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
+          <t>XXXXXX8441</t>
         </is>
       </c>
       <c r="E113" s="32" t="inlineStr">
@@ -7085,17 +7085,17 @@
       </c>
       <c r="H113" s="33" t="inlineStr">
         <is>
-          <t>Line 27</t>
+          <t>Line 160</t>
         </is>
       </c>
       <c r="I113" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J113" s="34" t="inlineStr">
         <is>
-          <t>From: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
+          <t>Consultant Contact NoXXXXXX8441</t>
         </is>
       </c>
     </row>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="D114" s="31" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E114" s="32" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="H114" s="30" t="inlineStr">
         <is>
-          <t>Line 29</t>
+          <t>Line 1</t>
         </is>
       </c>
       <c r="I114" s="31" t="inlineStr">
@@ -7145,7 +7145,7 @@
       </c>
       <c r="J114" s="31" t="inlineStr">
         <is>
-          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>From:"Parmod Kumar" &lt;i***d@sportking.co.in&gt;</t>
         </is>
       </c>
     </row>
@@ -7165,7 +7165,7 @@
       </c>
       <c r="D115" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>r***d@mawaimail.com</t>
         </is>
       </c>
       <c r="E115" s="32" t="inlineStr">
@@ -7185,7 +7185,7 @@
       </c>
       <c r="H115" s="33" t="inlineStr">
         <is>
-          <t>Line 30</t>
+          <t>Line 2</t>
         </is>
       </c>
       <c r="I115" s="34" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="J115" s="34" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>To: "Rahul Raj" &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="D116" s="31" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>r***d@mawaimail.com</t>
         </is>
       </c>
       <c r="E116" s="32" t="inlineStr">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="H116" s="30" t="inlineStr">
         <is>
-          <t>Line 30</t>
+          <t>Line 11</t>
         </is>
       </c>
       <c r="I116" s="31" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="J116" s="31" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="D117" s="34" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E117" s="32" t="inlineStr">
@@ -7285,7 +7285,7 @@
       </c>
       <c r="H117" s="33" t="inlineStr">
         <is>
-          <t>Line 36</t>
+          <t>Line 13</t>
         </is>
       </c>
       <c r="I117" s="34" t="inlineStr">
@@ -7295,7 +7295,7 @@
       </c>
       <c r="J117" s="34" t="inlineStr">
         <is>
-          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>To: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
         </is>
       </c>
     </row>
@@ -7315,7 +7315,7 @@
       </c>
       <c r="D118" s="31" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E118" s="32" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="H118" s="30" t="inlineStr">
         <is>
-          <t>Line 38</t>
+          <t>Line 14</t>
         </is>
       </c>
       <c r="I118" s="31" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="J118" s="31" t="inlineStr">
         <is>
-          <t>To: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7365,7 @@
       </c>
       <c r="D119" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>a***h@mawaimail.com</t>
         </is>
       </c>
       <c r="E119" s="32" t="inlineStr">
@@ -7385,7 +7385,7 @@
       </c>
       <c r="H119" s="33" t="inlineStr">
         <is>
-          <t>Line 39</t>
+          <t>Line 14</t>
         </is>
       </c>
       <c r="I119" s="34" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="J119" s="34" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="D120" s="31" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E120" s="32" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="H120" s="30" t="inlineStr">
         <is>
-          <t>Line 39</t>
+          <t>Line 27</t>
         </is>
       </c>
       <c r="I120" s="31" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="J120" s="31" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>From: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
         </is>
       </c>
     </row>
@@ -7460,12 +7460,12 @@
       </c>
       <c r="C121" s="33" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D121" s="34" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>r***d@mawaimail.com</t>
         </is>
       </c>
       <c r="E121" s="32" t="inlineStr">
@@ -7485,17 +7485,17 @@
       </c>
       <c r="H121" s="33" t="inlineStr">
         <is>
-          <t>Line 46</t>
+          <t>Line 29</t>
         </is>
       </c>
       <c r="I121" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J121" s="34" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7510,22 +7510,22 @@
       </c>
       <c r="C122" s="30" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D122" s="31" t="inlineStr">
         <is>
-          <t>20XX07</t>
-        </is>
-      </c>
-      <c r="E122" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>v***a@mawaimail.com</t>
+        </is>
+      </c>
+      <c r="E122" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F122" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G122" s="30" t="inlineStr">
@@ -7535,17 +7535,17 @@
       </c>
       <c r="H122" s="30" t="inlineStr">
         <is>
-          <t>Line 50</t>
+          <t>Line 30</t>
         </is>
       </c>
       <c r="I122" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J122" s="31" t="inlineStr">
         <is>
-          <t>20XX07- U.P</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="D123" s="34" t="inlineStr">
         <is>
-          <t>s***s@mawaimail.com</t>
+          <t>a***h@mawaimail.com</t>
         </is>
       </c>
       <c r="E123" s="32" t="inlineStr">
@@ -7585,7 +7585,7 @@
       </c>
       <c r="H123" s="33" t="inlineStr">
         <is>
-          <t>Line 52</t>
+          <t>Line 30</t>
         </is>
       </c>
       <c r="I123" s="34" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="J123" s="34" t="inlineStr">
         <is>
-          <t>From: SAP Access &lt;s***s@mawaimail.com&gt;</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7635,7 +7635,7 @@
       </c>
       <c r="H124" s="30" t="inlineStr">
         <is>
-          <t>Line 54</t>
+          <t>Line 36</t>
         </is>
       </c>
       <c r="I124" s="31" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="J124" s="31" t="inlineStr">
         <is>
-          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7665,7 +7665,7 @@
       </c>
       <c r="D125" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E125" s="32" t="inlineStr">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="H125" s="33" t="inlineStr">
         <is>
-          <t>Line 55</t>
+          <t>Line 38</t>
         </is>
       </c>
       <c r="I125" s="34" t="inlineStr">
@@ -7695,7 +7695,7 @@
       </c>
       <c r="J125" s="34" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>To: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
         </is>
       </c>
     </row>
@@ -7715,7 +7715,7 @@
       </c>
       <c r="D126" s="31" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E126" s="32" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="H126" s="30" t="inlineStr">
         <is>
-          <t>Line 55</t>
+          <t>Line 39</t>
         </is>
       </c>
       <c r="I126" s="31" t="inlineStr">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="J126" s="31" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7760,12 +7760,12 @@
       </c>
       <c r="C127" s="33" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D127" s="34" t="inlineStr">
         <is>
-          <t>XXXXXX7531</t>
+          <t>a***h@mawaimail.com</t>
         </is>
       </c>
       <c r="E127" s="32" t="inlineStr">
@@ -7785,17 +7785,17 @@
       </c>
       <c r="H127" s="33" t="inlineStr">
         <is>
-          <t>Line 61</t>
+          <t>Line 39</t>
         </is>
       </c>
       <c r="I127" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J127" s="34" t="inlineStr">
         <is>
-          <t>XXXXXX7531</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7810,22 +7810,22 @@
       </c>
       <c r="C128" s="30" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D128" s="31" t="inlineStr">
         <is>
-          <t>20XX01</t>
-        </is>
-      </c>
-      <c r="E128" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>s***s@mawaimail.com</t>
+        </is>
+      </c>
+      <c r="E128" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F128" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G128" s="30" t="inlineStr">
@@ -7835,17 +7835,17 @@
       </c>
       <c r="H128" s="30" t="inlineStr">
         <is>
-          <t>Line 65</t>
+          <t>Line 52</t>
         </is>
       </c>
       <c r="I128" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J128" s="31" t="inlineStr">
         <is>
-          <t>20XX01- U.P. (INDIA)</t>
+          <t>From: SAP Access &lt;s***s@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7885,7 +7885,7 @@
       </c>
       <c r="H129" s="33" t="inlineStr">
         <is>
-          <t>Line 67</t>
+          <t>Line 54</t>
         </is>
       </c>
       <c r="I129" s="34" t="inlineStr">
@@ -7895,7 +7895,7 @@
       </c>
       <c r="J129" s="34" t="inlineStr">
         <is>
-          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7915,7 +7915,7 @@
       </c>
       <c r="D130" s="31" t="inlineStr">
         <is>
-          <t>s***s@mawaimail.com</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E130" s="32" t="inlineStr">
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H130" s="30" t="inlineStr">
         <is>
-          <t>Line 69</t>
+          <t>Line 55</t>
         </is>
       </c>
       <c r="I130" s="31" t="inlineStr">
@@ -7945,7 +7945,7 @@
       </c>
       <c r="J130" s="31" t="inlineStr">
         <is>
-          <t>To: SAP Access &lt;s***s@mawaimail.com&gt;</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="D131" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>a***h@mawaimail.com</t>
         </is>
       </c>
       <c r="E131" s="32" t="inlineStr">
@@ -7985,7 +7985,7 @@
       </c>
       <c r="H131" s="33" t="inlineStr">
         <is>
-          <t>Line 70</t>
+          <t>Line 55</t>
         </is>
       </c>
       <c r="I131" s="34" t="inlineStr">
@@ -7995,7 +7995,7 @@
       </c>
       <c r="J131" s="34" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="D132" s="31" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>r***d@mawaimail.com</t>
         </is>
       </c>
       <c r="E132" s="32" t="inlineStr">
@@ -8035,7 +8035,7 @@
       </c>
       <c r="H132" s="30" t="inlineStr">
         <is>
-          <t>Line 70</t>
+          <t>Line 67</t>
         </is>
       </c>
       <c r="I132" s="31" t="inlineStr">
@@ -8045,7 +8045,7 @@
       </c>
       <c r="J132" s="31" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8060,22 +8060,22 @@
       </c>
       <c r="C133" s="33" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D133" s="34" t="inlineStr">
         <is>
-          <t>90XX53</t>
-        </is>
-      </c>
-      <c r="E133" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>s***s@mawaimail.com</t>
+        </is>
+      </c>
+      <c r="E133" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F133" s="33" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G133" s="33" t="inlineStr">
@@ -8085,17 +8085,17 @@
       </c>
       <c r="H133" s="33" t="inlineStr">
         <is>
-          <t>Line 74</t>
+          <t>Line 69</t>
         </is>
       </c>
       <c r="I133" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J133" s="34" t="inlineStr">
         <is>
-          <t>he TR from DEV to QAS  (Sportking), SKDK90XX53              ABAPCONS ZSCN Validity</t>
+          <t>To: SAP Access &lt;s***s@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8110,12 +8110,12 @@
       </c>
       <c r="C134" s="30" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D134" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E134" s="32" t="inlineStr">
@@ -8135,17 +8135,17 @@
       </c>
       <c r="H134" s="30" t="inlineStr">
         <is>
-          <t>Line 78</t>
+          <t>Line 70</t>
         </is>
       </c>
       <c r="I134" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J134" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8160,22 +8160,22 @@
       </c>
       <c r="C135" s="33" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D135" s="34" t="inlineStr">
         <is>
-          <t>20XX07</t>
-        </is>
-      </c>
-      <c r="E135" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>a***h@mawaimail.com</t>
+        </is>
+      </c>
+      <c r="E135" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F135" s="33" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G135" s="33" t="inlineStr">
@@ -8185,17 +8185,17 @@
       </c>
       <c r="H135" s="33" t="inlineStr">
         <is>
-          <t>Line 82</t>
+          <t>Line 70</t>
         </is>
       </c>
       <c r="I135" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J135" s="34" t="inlineStr">
         <is>
-          <t>20XX07- U.P</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8610,12 +8610,12 @@
       </c>
       <c r="C144" s="30" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D144" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E144" s="32" t="inlineStr">
@@ -8635,17 +8635,17 @@
       </c>
       <c r="H144" s="30" t="inlineStr">
         <is>
-          <t>Line 103</t>
+          <t>Line 109</t>
         </is>
       </c>
       <c r="I144" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J144" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>From: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
         </is>
       </c>
     </row>
@@ -8660,22 +8660,22 @@
       </c>
       <c r="C145" s="33" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D145" s="34" t="inlineStr">
         <is>
-          <t>20XX07</t>
-        </is>
-      </c>
-      <c r="E145" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>r***d@mawaimail.com</t>
+        </is>
+      </c>
+      <c r="E145" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F145" s="33" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G145" s="33" t="inlineStr">
@@ -8685,17 +8685,17 @@
       </c>
       <c r="H145" s="33" t="inlineStr">
         <is>
-          <t>Line 107</t>
+          <t>Line 111</t>
         </is>
       </c>
       <c r="I145" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J145" s="34" t="inlineStr">
         <is>
-          <t>20XX07- U.P</t>
+          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8715,7 @@
       </c>
       <c r="D146" s="31" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E146" s="32" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="H146" s="30" t="inlineStr">
         <is>
-          <t>Line 109</t>
+          <t>Line 112</t>
         </is>
       </c>
       <c r="I146" s="31" t="inlineStr">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="J146" s="31" t="inlineStr">
         <is>
-          <t>From: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8765,7 +8765,7 @@
       </c>
       <c r="D147" s="34" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>a***h@mawaimail.com</t>
         </is>
       </c>
       <c r="E147" s="32" t="inlineStr">
@@ -8785,7 +8785,7 @@
       </c>
       <c r="H147" s="33" t="inlineStr">
         <is>
-          <t>Line 111</t>
+          <t>Line 112</t>
         </is>
       </c>
       <c r="I147" s="34" t="inlineStr">
@@ -8795,7 +8795,7 @@
       </c>
       <c r="J147" s="34" t="inlineStr">
         <is>
-          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8815,7 +8815,7 @@
       </c>
       <c r="D148" s="31" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>r***d@mawaimail.com</t>
         </is>
       </c>
       <c r="E148" s="32" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="H148" s="30" t="inlineStr">
         <is>
-          <t>Line 112</t>
+          <t>Line 120</t>
         </is>
       </c>
       <c r="I148" s="31" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="J148" s="31" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8865,7 +8865,7 @@
       </c>
       <c r="D149" s="34" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E149" s="32" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="H149" s="33" t="inlineStr">
         <is>
-          <t>Line 112</t>
+          <t>Line 122</t>
         </is>
       </c>
       <c r="I149" s="34" t="inlineStr">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="J149" s="34" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>To: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
         </is>
       </c>
     </row>
@@ -8910,12 +8910,12 @@
       </c>
       <c r="C150" s="30" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D150" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8277</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E150" s="32" t="inlineStr">
@@ -8935,17 +8935,17 @@
       </c>
       <c r="H150" s="30" t="inlineStr">
         <is>
-          <t>Line 119</t>
+          <t>Line 123</t>
         </is>
       </c>
       <c r="I150" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J150" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8277</t>
+          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="D151" s="34" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>a***h@mawaimail.com</t>
         </is>
       </c>
       <c r="E151" s="32" t="inlineStr">
@@ -8985,7 +8985,7 @@
       </c>
       <c r="H151" s="33" t="inlineStr">
         <is>
-          <t>Line 120</t>
+          <t>Line 123</t>
         </is>
       </c>
       <c r="I151" s="34" t="inlineStr">
@@ -8995,7 +8995,7 @@
       </c>
       <c r="J151" s="34" t="inlineStr">
         <is>
-          <t>From: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="D152" s="31" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
+          <t>n***y@mawaimail.com</t>
         </is>
       </c>
       <c r="E152" s="32" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="H152" s="30" t="inlineStr">
         <is>
-          <t>Line 122</t>
+          <t>Line 138</t>
         </is>
       </c>
       <c r="I152" s="31" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="J152" s="31" t="inlineStr">
         <is>
-          <t>To: Parmod Kumar &lt;i***d@sportking.co.in&gt;</t>
+          <t>From: No reply &lt;n***y@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -9065,7 +9065,7 @@
       </c>
       <c r="D153" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>r***d@mawaimail.com</t>
         </is>
       </c>
       <c r="E153" s="32" t="inlineStr">
@@ -9085,7 +9085,7 @@
       </c>
       <c r="H153" s="33" t="inlineStr">
         <is>
-          <t>Line 123</t>
+          <t>Line 140</t>
         </is>
       </c>
       <c r="I153" s="34" t="inlineStr">
@@ -9095,7 +9095,7 @@
       </c>
       <c r="J153" s="34" t="inlineStr">
         <is>
-          <t>Cc: Vanshika Shukla &lt;v***a@mawaimail.com&gt;; Akash Tripathi &lt;akash@mawaimail.com&gt;</t>
+          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -9115,7 +9115,7 @@
       </c>
       <c r="D154" s="31" t="inlineStr">
         <is>
-          <t>a***h@mawaimail.com</t>
+          <t>s***t@mawaimail.com</t>
         </is>
       </c>
       <c r="E154" s="32" t="inlineStr">
@@ -9135,7 +9135,7 @@
       </c>
       <c r="H154" s="30" t="inlineStr">
         <is>
-          <t>Line 123</t>
+          <t>Line 141</t>
         </is>
       </c>
       <c r="I154" s="31" t="inlineStr">
@@ -9145,7 +9145,7 @@
       </c>
       <c r="J154" s="31" t="inlineStr">
         <is>
-          <t>anshika@mawaimail.com&gt;; Akash Tripathi &lt;a***h@mawaimail.com&gt;</t>
+          <t>Cc: Sap Support &lt;s***t@mawaimail.com&gt;;sdsupport@mawaimail.com &lt;sdsupport@maw</t>
         </is>
       </c>
     </row>
@@ -9160,12 +9160,12 @@
       </c>
       <c r="C155" s="33" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D155" s="34" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>s***t@mawaimail.com</t>
         </is>
       </c>
       <c r="E155" s="32" t="inlineStr">
@@ -9185,17 +9185,17 @@
       </c>
       <c r="H155" s="33" t="inlineStr">
         <is>
-          <t>Line 132</t>
+          <t>Line 141</t>
         </is>
       </c>
       <c r="I155" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J155" s="34" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
+          <t>Sap Support &lt;sapsupport@mawaimail.com&gt;;s***t@mawaimail.com &lt;s***t@mawaimail.com&gt;; Vika</t>
         </is>
       </c>
     </row>
@@ -9210,22 +9210,22 @@
       </c>
       <c r="C156" s="30" t="inlineStr">
         <is>
-          <t>PIN_CODE</t>
+          <t>EMAIL</t>
         </is>
       </c>
       <c r="D156" s="31" t="inlineStr">
         <is>
-          <t>20XX07</t>
-        </is>
-      </c>
-      <c r="E156" s="35" t="inlineStr">
-        <is>
-          <t>LOW</t>
+          <t>v***a@mawaimail.com</t>
+        </is>
+      </c>
+      <c r="E156" s="32" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="F156" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="G156" s="30" t="inlineStr">
@@ -9235,17 +9235,17 @@
       </c>
       <c r="H156" s="30" t="inlineStr">
         <is>
-          <t>Line 136</t>
+          <t>Line 142</t>
         </is>
       </c>
       <c r="I156" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023 (location data when linked to address)</t>
+          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
         </is>
       </c>
       <c r="J156" s="31" t="inlineStr">
         <is>
-          <t>20XX07- U.P</t>
+          <t>Gupta &lt;v***a@mawaimail.com&gt;; Shivani Mishra &lt;shivani@mawaimail.com</t>
         </is>
       </c>
     </row>
@@ -9265,7 +9265,7 @@
       </c>
       <c r="D157" s="34" t="inlineStr">
         <is>
-          <t>n***y@mawaimail.com</t>
+          <t>s***i@mawaimail.com</t>
         </is>
       </c>
       <c r="E157" s="32" t="inlineStr">
@@ -9285,7 +9285,7 @@
       </c>
       <c r="H157" s="33" t="inlineStr">
         <is>
-          <t>Line 138</t>
+          <t>Line 142</t>
         </is>
       </c>
       <c r="I157" s="34" t="inlineStr">
@@ -9295,7 +9295,7 @@
       </c>
       <c r="J157" s="34" t="inlineStr">
         <is>
-          <t>From: No reply &lt;n***y@mawaimail.com&gt;</t>
+          <t>a &lt;vika@mawaimail.com&gt;; Shivani Mishra &lt;s***i@mawaimail.com&gt;; Vanshika Shukla</t>
         </is>
       </c>
     </row>
@@ -9315,7 +9315,7 @@
       </c>
       <c r="D158" s="31" t="inlineStr">
         <is>
-          <t>r***d@mawaimail.com</t>
+          <t>v***a@mawaimail.com</t>
         </is>
       </c>
       <c r="E158" s="32" t="inlineStr">
@@ -9335,7 +9335,7 @@
       </c>
       <c r="H158" s="30" t="inlineStr">
         <is>
-          <t>Line 140</t>
+          <t>Line 143</t>
         </is>
       </c>
       <c r="I158" s="31" t="inlineStr">
@@ -9345,7 +9345,7 @@
       </c>
       <c r="J158" s="31" t="inlineStr">
         <is>
-          <t>To: Rahul Raj &lt;r***d@mawaimail.com&gt;</t>
+          <t>&lt;v***a@mawaimail.com&gt;; Debashree Sarkar &lt;debashree@mawaimail</t>
         </is>
       </c>
     </row>
@@ -9365,7 +9365,7 @@
       </c>
       <c r="D159" s="34" t="inlineStr">
         <is>
-          <t>s***t@mawaimail.com</t>
+          <t>d***e@mawaimail.com</t>
         </is>
       </c>
       <c r="E159" s="32" t="inlineStr">
@@ -9385,7 +9385,7 @@
       </c>
       <c r="H159" s="33" t="inlineStr">
         <is>
-          <t>Line 141</t>
+          <t>Line 143</t>
         </is>
       </c>
       <c r="I159" s="34" t="inlineStr">
@@ -9395,7 +9395,7 @@
       </c>
       <c r="J159" s="34" t="inlineStr">
         <is>
-          <t>Cc: Sap Support &lt;s***t@mawaimail.com&gt;;sdsupport@mawaimail.com &lt;sdsupport@maw</t>
+          <t>shika@mawaimail.com&gt;; Debashree Sarkar &lt;d***e@mawaimail.com&gt;; Megha Yadav</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9415,7 @@
       </c>
       <c r="D160" s="31" t="inlineStr">
         <is>
-          <t>s***t@mawaimail.com</t>
+          <t>m***v@mawaimail.com</t>
         </is>
       </c>
       <c r="E160" s="32" t="inlineStr">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="H160" s="30" t="inlineStr">
         <is>
-          <t>Line 141</t>
+          <t>Line 144</t>
         </is>
       </c>
       <c r="I160" s="31" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="J160" s="31" t="inlineStr">
         <is>
-          <t>Sap Support &lt;sapsupport@mawaimail.com&gt;;s***t@mawaimail.com &lt;s***t@mawaimail.com&gt;; Vika</t>
+          <t>&lt;m***v@mawaimail.com&gt;</t>
         </is>
       </c>
     </row>
@@ -9465,7 +9465,7 @@
       </c>
       <c r="D161" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
+          <t>i***d@sportking.co.in</t>
         </is>
       </c>
       <c r="E161" s="32" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="H161" s="33" t="inlineStr">
         <is>
-          <t>Line 142</t>
+          <t>Line 157</t>
         </is>
       </c>
       <c r="I161" s="34" t="inlineStr">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="J161" s="34" t="inlineStr">
         <is>
-          <t>Gupta &lt;v***a@mawaimail.com&gt;; Shivani Mishra &lt;shivani@mawaimail.com</t>
+          <t>Email Id i***d@sportking.co.in</t>
         </is>
       </c>
     </row>
@@ -9510,22 +9510,22 @@
       </c>
       <c r="C162" s="30" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D162" s="31" t="inlineStr">
         <is>
-          <t>s***i@mawaimail.com</t>
-        </is>
-      </c>
-      <c r="E162" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>20XX07</t>
+        </is>
+      </c>
+      <c r="E162" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F162" s="30" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G162" s="30" t="inlineStr">
@@ -9535,17 +9535,17 @@
       </c>
       <c r="H162" s="30" t="inlineStr">
         <is>
-          <t>Line 142</t>
+          <t>Line 25</t>
         </is>
       </c>
       <c r="I162" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J162" s="31" t="inlineStr">
         <is>
-          <t>a &lt;vika@mawaimail.com&gt;; Shivani Mishra &lt;s***i@mawaimail.com&gt;; Vanshika Shukla</t>
+          <t>20XX07- U.P</t>
         </is>
       </c>
     </row>
@@ -9560,22 +9560,22 @@
       </c>
       <c r="C163" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D163" s="34" t="inlineStr">
         <is>
-          <t>v***a@mawaimail.com</t>
-        </is>
-      </c>
-      <c r="E163" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>20XX07</t>
+        </is>
+      </c>
+      <c r="E163" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F163" s="33" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G163" s="33" t="inlineStr">
@@ -9585,17 +9585,17 @@
       </c>
       <c r="H163" s="33" t="inlineStr">
         <is>
-          <t>Line 143</t>
+          <t>Line 50</t>
         </is>
       </c>
       <c r="I163" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J163" s="34" t="inlineStr">
         <is>
-          <t>&lt;v***a@mawaimail.com&gt;; Debashree Sarkar &lt;debashree@mawaimail</t>
+          <t>20XX07- U.P</t>
         </is>
       </c>
     </row>
@@ -9610,22 +9610,22 @@
       </c>
       <c r="C164" s="30" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D164" s="31" t="inlineStr">
         <is>
-          <t>d***e@mawaimail.com</t>
-        </is>
-      </c>
-      <c r="E164" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>20XX01</t>
+        </is>
+      </c>
+      <c r="E164" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F164" s="30" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G164" s="30" t="inlineStr">
@@ -9635,17 +9635,17 @@
       </c>
       <c r="H164" s="30" t="inlineStr">
         <is>
-          <t>Line 143</t>
+          <t>Line 65</t>
         </is>
       </c>
       <c r="I164" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J164" s="31" t="inlineStr">
         <is>
-          <t>shika@mawaimail.com&gt;; Debashree Sarkar &lt;d***e@mawaimail.com&gt;; Megha Yadav</t>
+          <t>20XX01- U.P. (INDIA)</t>
         </is>
       </c>
     </row>
@@ -9660,22 +9660,22 @@
       </c>
       <c r="C165" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D165" s="34" t="inlineStr">
         <is>
-          <t>m***v@mawaimail.com</t>
-        </is>
-      </c>
-      <c r="E165" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>90XX53</t>
+        </is>
+      </c>
+      <c r="E165" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F165" s="33" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G165" s="33" t="inlineStr">
@@ -9685,17 +9685,17 @@
       </c>
       <c r="H165" s="33" t="inlineStr">
         <is>
-          <t>Line 144</t>
+          <t>Line 74</t>
         </is>
       </c>
       <c r="I165" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J165" s="34" t="inlineStr">
         <is>
-          <t>&lt;m***v@mawaimail.com&gt;</t>
+          <t>he TR from DEV to QAS  (Sportking), SKDK90XX53              ABAPCONS ZSCN Validity</t>
         </is>
       </c>
     </row>
@@ -9710,22 +9710,22 @@
       </c>
       <c r="C166" s="30" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D166" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8277</t>
-        </is>
-      </c>
-      <c r="E166" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>20XX07</t>
+        </is>
+      </c>
+      <c r="E166" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F166" s="30" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G166" s="30" t="inlineStr">
@@ -9735,17 +9735,17 @@
       </c>
       <c r="H166" s="30" t="inlineStr">
         <is>
-          <t>Line 156</t>
+          <t>Line 82</t>
         </is>
       </c>
       <c r="I166" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J166" s="31" t="inlineStr">
         <is>
-          <t>Phone Number XXXXXX8277</t>
+          <t>20XX07- U.P</t>
         </is>
       </c>
     </row>
@@ -9760,22 +9760,22 @@
       </c>
       <c r="C167" s="33" t="inlineStr">
         <is>
-          <t>EMAIL</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D167" s="34" t="inlineStr">
         <is>
-          <t>i***d@sportking.co.in</t>
-        </is>
-      </c>
-      <c r="E167" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>20XX07</t>
+        </is>
+      </c>
+      <c r="E167" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F167" s="33" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G167" s="33" t="inlineStr">
@@ -9785,17 +9785,17 @@
       </c>
       <c r="H167" s="33" t="inlineStr">
         <is>
-          <t>Line 157</t>
+          <t>Line 107</t>
         </is>
       </c>
       <c r="I167" s="34" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, IT Rules 2011 Sec 3, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J167" s="34" t="inlineStr">
         <is>
-          <t>Email Id i***d@sportking.co.in</t>
+          <t>20XX07- U.P</t>
         </is>
       </c>
     </row>
@@ -9810,22 +9810,22 @@
       </c>
       <c r="C168" s="30" t="inlineStr">
         <is>
-          <t>PHONE_IN</t>
+          <t>PIN_CODE</t>
         </is>
       </c>
       <c r="D168" s="31" t="inlineStr">
         <is>
-          <t>XXXXXX8441</t>
-        </is>
-      </c>
-      <c r="E168" s="32" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+          <t>20XX07</t>
+        </is>
+      </c>
+      <c r="E168" s="35" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F168" s="30" t="inlineStr">
         <is>
-          <t>85%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G168" s="30" t="inlineStr">
@@ -9835,17 +9835,17 @@
       </c>
       <c r="H168" s="30" t="inlineStr">
         <is>
-          <t>Line 160</t>
+          <t>Line 136</t>
         </is>
       </c>
       <c r="I168" s="31" t="inlineStr">
         <is>
-          <t>DPDP Act 2023, TRAI Privacy Regulations, DPDP Rules 2025</t>
+          <t>DPDP Act 2023 (location data when linked to address)</t>
         </is>
       </c>
       <c r="J168" s="31" t="inlineStr">
         <is>
-          <t>Consultant Contact NoXXXXXX8441</t>
+          <t>20XX07- U.P</t>
         </is>
       </c>
     </row>

</xml_diff>